<commit_message>
chore: include trial reports and upload sheet mapping verification tests
</commit_message>
<xml_diff>
--- a/Radiance_MC03_Daily_Trial_Review_2026-09-17.xlsx
+++ b/Radiance_MC03_Daily_Trial_Review_2026-09-17.xlsx
@@ -31,28 +31,38 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -61,13 +71,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -400,176 +412,176 @@
   <dimension ref="A1:C18"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" s="2" t="str">
         <v>RADIANCE POLYMERS PVT. LTD. - DAILY TRIAL REVIEW SUMMARY (MC03)</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2" s="2" t="str">
         <v>Generated Date:</v>
       </c>
-      <c r="B2" t="str">
-        <v>17/9/2026, 12:26:38 pm</v>
+      <c r="B2" s="2" t="str">
+        <v>4/10/2026, 11:51:43 am</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3" s="2" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4" s="2" t="str">
         <v>PARAMETER</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B4" s="2" t="str">
         <v>DAILY TRIAL RECORD</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C4" s="2" t="str">
         <v>BENCHMARK / STATUS</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5" s="2" t="str">
         <v>Machine Code</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B5" s="2" t="str">
         <v>MC03</v>
       </c>
-      <c r="C5" t="str">
-        <v>KraussMaffei 250T</v>
+      <c r="C5" s="2" t="str">
+        <v>Milacron 450T</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
+      <c r="A6" s="2" t="str">
         <v>Part Number / Tool</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B6" s="2" t="str">
         <v>F53200000A</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C6" s="2" t="str">
         <v>Lower Housing (Active Pilot)</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
+      <c r="A7" s="2" t="str">
         <v>Floor Operator</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B7" s="2" t="str">
         <v>Ramesh</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C7" s="2" t="str">
         <v>Floor Traceability Verified</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
+      <c r="A8" s="2" t="str">
         <v>Shift Supervisor</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B8" s="2" t="str">
         <v>Mr. Lokesh</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C8" s="2" t="str">
         <v>Authorized Supervisor</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
+      <c r="A9" s="2" t="str">
         <v>Gross Production</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B9" s="2" t="str">
         <v>3,335 pcs</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C9" s="2" t="str">
         <v>Hourly Cycle Target Achieved</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
+      <c r="A10" s="2" t="str">
         <v>Accepted Production</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B10" s="2" t="str">
         <v>3,270 pcs</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C10" s="2" t="str">
         <v>98.05% Quality Yield</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
+      <c r="A11" s="2" t="str">
         <v>Rejections Logged</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B11" s="2" t="str">
         <v>65 pcs</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C11" s="2" t="str">
         <v>1.95% Rejection Rate (PASS)</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
+      <c r="A12" s="2" t="str">
         <v>Downtime Minutes</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B12" s="2" t="str">
         <v>60 mins</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C12" s="2" t="str">
         <v>Mould Cleaning &amp; Start-up</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
+      <c r="A13" s="2" t="str">
         <v>Material Consumption</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B13" s="2" t="str">
         <v>179.5 kg</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C13" s="2" t="str">
         <v>Gram Weight Conformance Verified</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="str">
+      <c r="A14" s="2" t="str">
         <v>Validation Errors Prevented</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B14" s="2" t="str">
         <v>24 Prevented</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C14" s="2" t="str">
         <v>Zero Non-Conforming Entries</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="str">
+      <c r="A15" s="2" t="str">
         <v>Issues Raised Today</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B15" s="2" t="str">
         <v>3 Logged</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15" s="2" t="str">
         <v>Continuous Floor Tracking</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="str">
+      <c r="A16" s="2" t="str">
         <v>Issues Closed Today</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B16" s="2" t="str">
         <v>3 Closed</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C16" s="2" t="str">
         <v>100% Closure Rate</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="str">
+      <c r="A17" s="2" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="str">
+      <c r="A18" s="2" t="str">
         <v>DAILY TRIAL STATUS:</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B18" s="2" t="str">
         <v>OPERATIONAL &amp; HEALTHY - MC03 TRIAL STABILIZED</v>
       </c>
     </row>

</xml_diff>